<commit_message>
Fix: Sprint 1: Mejoras Sprint 2
</commit_message>
<xml_diff>
--- a/DOCUMENTACION - APLI 2/Historias de usuario, historias técnicas y Pila del Producto.xlsx
+++ b/DOCUMENTACION - APLI 2/Historias de usuario, historias técnicas y Pila del Producto.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\stive\Documents\stiven\8 Semestre\Aplicaciones Informaticas II\Tareas Individuales\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E35170D4-3CEB-4249-A196-D2B4BB7BBDF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E912F745-8877-4280-B554-249A387EDC05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-19320" yWindow="-120" windowWidth="19440" windowHeight="14880" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Historias de Usuario" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="163">
   <si>
     <t>ID</t>
   </si>
@@ -370,9 +370,6 @@
     <t>Login funcional; validación de credenciales; sesiones activas correctamente; cierre de sesión operativo; acceso restringido según rol.</t>
   </si>
   <si>
-    <t>Desarrollo de API para gestión de usuarios</t>
-  </si>
-  <si>
     <t>Implementar endpoints y lógica de backend para registrar, consultar, actualizar, activar o desactivar usuarios.</t>
   </si>
   <si>
@@ -388,9 +385,6 @@
     <t>Formularios funcionales; listado de usuarios visible; edición operativa; mensajes de confirmación y error mostrados correctamente.</t>
   </si>
   <si>
-    <t>Desarrollo de API para asistencias, horarios y pagos</t>
-  </si>
-  <si>
     <t>Implementar endpoints para registrar asistencias, gestionar horarios y registrar pagos de atletas.</t>
   </si>
   <si>
@@ -521,6 +515,18 @@
   </si>
   <si>
     <t>Implementación del módulo de evaluaciones</t>
+  </si>
+  <si>
+    <t>Implementación del módulo de gestión de usuarios</t>
+  </si>
+  <si>
+    <t>Implementación del módulo de asistencias, horarios y pagos</t>
+  </si>
+  <si>
+    <t>Desarrollo del modulo para asistencias, horarios y pagos</t>
+  </si>
+  <si>
+    <t>Desarrollo del modulo  para gestión de usuarios</t>
   </si>
 </sst>
 </file>
@@ -665,30 +671,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -703,6 +685,30 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -999,17 +1005,17 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7"/>
-      <c r="I2" s="7"/>
-      <c r="J2" s="8"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
+      <c r="H2" s="16"/>
+      <c r="I2" s="16"/>
+      <c r="J2" s="17"/>
     </row>
     <row r="3" spans="2:10" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B3" s="2" t="s">
@@ -1301,7 +1307,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="2:10" s="14" customFormat="1" ht="104.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:10" s="6" customFormat="1" ht="104.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="1" t="s">
         <v>99</v>
       </c>
@@ -1331,20 +1337,20 @@
       </c>
     </row>
     <row r="14" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B14" s="9" t="s">
+      <c r="B14" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="C14" s="9"/>
-      <c r="D14" s="9"/>
-      <c r="E14" s="9"/>
-      <c r="F14" s="9"/>
-      <c r="G14" s="9"/>
-      <c r="H14" s="9"/>
-      <c r="I14" s="9">
+      <c r="C14" s="18"/>
+      <c r="D14" s="18"/>
+      <c r="E14" s="18"/>
+      <c r="F14" s="18"/>
+      <c r="G14" s="18"/>
+      <c r="H14" s="18"/>
+      <c r="I14" s="18">
         <f>SUM(I4:I13)</f>
         <v>44</v>
       </c>
-      <c r="J14" s="9"/>
+      <c r="J14" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -1371,492 +1377,492 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
-      <c r="H2" s="18"/>
-      <c r="I2" s="18"/>
-      <c r="J2" s="19"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
+      <c r="G2" s="10"/>
+      <c r="H2" s="10"/>
+      <c r="I2" s="10"/>
+      <c r="J2" s="11"/>
     </row>
     <row r="3" spans="2:10" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="B3" s="15" t="s">
+      <c r="B3" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="15" t="s">
+      <c r="C3" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="D3" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="15" t="s">
+      <c r="E3" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="F3" s="15" t="s">
+      <c r="F3" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="G3" s="15" t="s">
+      <c r="G3" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="H3" s="15" t="s">
+      <c r="H3" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="I3" s="15" t="s">
+      <c r="I3" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="J3" s="15" t="s">
+      <c r="J3" s="7" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="4" spans="2:10" ht="204.75" x14ac:dyDescent="0.25">
-      <c r="B4" s="16" t="s">
+      <c r="B4" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="C4" s="16" t="s">
+      <c r="C4" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="D4" s="16" t="s">
+      <c r="D4" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="E4" s="16" t="s">
+      <c r="E4" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="F4" s="16" t="s">
+      <c r="F4" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="G4" s="16" t="s">
-        <v>8</v>
-      </c>
-      <c r="H4" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="I4" s="16">
+      <c r="G4" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="I4" s="8">
         <v>3</v>
       </c>
-      <c r="J4" s="16" t="s">
+      <c r="J4" s="8" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="5" spans="2:10" ht="126" x14ac:dyDescent="0.25">
-      <c r="B5" s="16" t="s">
+      <c r="B5" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="C5" s="16" t="s">
+      <c r="C5" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D5" s="16" t="s">
+      <c r="D5" s="8" t="s">
         <v>108</v>
       </c>
-      <c r="E5" s="16" t="s">
+      <c r="E5" s="8" t="s">
         <v>109</v>
       </c>
-      <c r="F5" s="16" t="s">
+      <c r="F5" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="G5" s="16" t="s">
-        <v>8</v>
-      </c>
-      <c r="H5" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="I5" s="16">
+      <c r="G5" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="H5" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="I5" s="8">
         <v>3</v>
       </c>
-      <c r="J5" s="16" t="s">
+      <c r="J5" s="8" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="6" spans="2:10" ht="126" x14ac:dyDescent="0.25">
-      <c r="B6" s="16" t="s">
+      <c r="B6" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="C6" s="16" t="s">
+      <c r="C6" s="8" t="s">
+        <v>159</v>
+      </c>
+      <c r="D6" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="D6" s="16" t="s">
+      <c r="E6" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="E6" s="16" t="s">
+      <c r="F6" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="G6" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="H6" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="I6" s="8">
+        <v>3</v>
+      </c>
+      <c r="J6" s="8" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="2:10" ht="94.5" x14ac:dyDescent="0.25">
+      <c r="B7" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="C7" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="F6" s="16" t="s">
+      <c r="D7" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="F7" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="G6" s="16" t="s">
-        <v>8</v>
-      </c>
-      <c r="H6" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="I6" s="16">
+      <c r="G7" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="I7" s="8">
         <v>3</v>
       </c>
-      <c r="J6" s="16" t="s">
+      <c r="J7" s="8" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="2:10" ht="94.5" x14ac:dyDescent="0.25">
-      <c r="B7" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="C7" s="16" t="s">
-        <v>113</v>
-      </c>
-      <c r="D7" s="16" t="s">
-        <v>114</v>
-      </c>
-      <c r="E7" s="16" t="s">
+    <row r="8" spans="2:10" ht="110.25" x14ac:dyDescent="0.25">
+      <c r="B8" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>160</v>
+      </c>
+      <c r="D8" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="F7" s="16" t="s">
-        <v>47</v>
-      </c>
-      <c r="G7" s="16" t="s">
-        <v>8</v>
-      </c>
-      <c r="H7" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="I7" s="16">
+      <c r="E8" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="G8" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="H8" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="I8" s="8">
+        <v>4</v>
+      </c>
+      <c r="J8" s="8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="2:10" ht="110.25" x14ac:dyDescent="0.25">
+      <c r="B9" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="G9" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="H9" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="I9" s="8">
+        <v>5</v>
+      </c>
+      <c r="J9" s="8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="2:10" ht="126" x14ac:dyDescent="0.25">
+      <c r="B10" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="G10" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="H10" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="I10" s="8">
+        <v>5</v>
+      </c>
+      <c r="J10" s="8" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11" spans="2:10" ht="94.5" x14ac:dyDescent="0.25">
+      <c r="B11" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="G11" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="H11" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="I11" s="8">
+        <v>4</v>
+      </c>
+      <c r="J11" s="8" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="12" spans="2:10" ht="141.75" x14ac:dyDescent="0.25">
+      <c r="B12" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="G12" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="H12" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="I12" s="8">
+        <v>6</v>
+      </c>
+      <c r="J12" s="8" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="13" spans="2:10" ht="157.5" x14ac:dyDescent="0.25">
+      <c r="B13" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>132</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="G13" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="H13" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="I13" s="8">
+        <v>4</v>
+      </c>
+      <c r="J13" s="8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="14" spans="2:10" ht="126" x14ac:dyDescent="0.25">
+      <c r="B14" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>136</v>
+      </c>
+      <c r="E14" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="G14" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="H14" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="I14" s="8">
+        <v>5</v>
+      </c>
+      <c r="J14" s="8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15" spans="2:10" ht="126" x14ac:dyDescent="0.25">
+      <c r="B15" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>140</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="F15" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="G15" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="H15" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="I15" s="8">
+        <v>4</v>
+      </c>
+      <c r="J15" s="8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="16" spans="2:10" ht="110.25" x14ac:dyDescent="0.25">
+      <c r="B16" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="F16" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="G16" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="H16" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="I16" s="8">
         <v>3</v>
       </c>
-      <c r="J7" s="16" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="8" spans="2:10" ht="110.25" x14ac:dyDescent="0.25">
-      <c r="B8" s="16" t="s">
-        <v>33</v>
-      </c>
-      <c r="C8" s="16" t="s">
-        <v>116</v>
-      </c>
-      <c r="D8" s="16" t="s">
-        <v>117</v>
-      </c>
-      <c r="E8" s="16" t="s">
-        <v>118</v>
-      </c>
-      <c r="F8" s="16" t="s">
-        <v>119</v>
-      </c>
-      <c r="G8" s="16" t="s">
-        <v>8</v>
-      </c>
-      <c r="H8" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="I8" s="16">
+      <c r="J16" s="8" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="17" spans="2:10" ht="110.25" x14ac:dyDescent="0.25">
+      <c r="B17" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="C17" s="8" t="s">
+        <v>147</v>
+      </c>
+      <c r="D17" s="8" t="s">
+        <v>148</v>
+      </c>
+      <c r="E17" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="F17" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="G17" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="H17" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="I17" s="8">
+        <v>5</v>
+      </c>
+      <c r="J17" s="8" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="18" spans="2:10" ht="126" x14ac:dyDescent="0.25">
+      <c r="B18" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>151</v>
+      </c>
+      <c r="D18" s="8" t="s">
+        <v>152</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="G18" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="H18" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="I18" s="8">
         <v>4</v>
       </c>
-      <c r="J8" s="16" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="9" spans="2:10" ht="110.25" x14ac:dyDescent="0.25">
-      <c r="B9" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="C9" s="16" t="s">
-        <v>120</v>
-      </c>
-      <c r="D9" s="16" t="s">
-        <v>121</v>
-      </c>
-      <c r="E9" s="16" t="s">
-        <v>122</v>
-      </c>
-      <c r="F9" s="16" t="s">
-        <v>123</v>
-      </c>
-      <c r="G9" s="16" t="s">
-        <v>8</v>
-      </c>
-      <c r="H9" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="I9" s="16">
-        <v>5</v>
-      </c>
-      <c r="J9" s="16" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="10" spans="2:10" ht="126" x14ac:dyDescent="0.25">
-      <c r="B10" s="16" t="s">
-        <v>35</v>
-      </c>
-      <c r="C10" s="16" t="s">
-        <v>124</v>
-      </c>
-      <c r="D10" s="16" t="s">
-        <v>125</v>
-      </c>
-      <c r="E10" s="16" t="s">
-        <v>126</v>
-      </c>
-      <c r="F10" s="16" t="s">
-        <v>87</v>
-      </c>
-      <c r="G10" s="16" t="s">
-        <v>8</v>
-      </c>
-      <c r="H10" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="I10" s="16">
-        <v>5</v>
-      </c>
-      <c r="J10" s="16" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="11" spans="2:10" ht="94.5" x14ac:dyDescent="0.25">
-      <c r="B11" s="16" t="s">
-        <v>36</v>
-      </c>
-      <c r="C11" s="16" t="s">
-        <v>57</v>
-      </c>
-      <c r="D11" s="16" t="s">
-        <v>127</v>
-      </c>
-      <c r="E11" s="16" t="s">
-        <v>128</v>
-      </c>
-      <c r="F11" s="16" t="s">
-        <v>106</v>
-      </c>
-      <c r="G11" s="16" t="s">
-        <v>8</v>
-      </c>
-      <c r="H11" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="I11" s="16">
-        <v>4</v>
-      </c>
-      <c r="J11" s="16" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="12" spans="2:10" ht="141.75" x14ac:dyDescent="0.25">
-      <c r="B12" s="16" t="s">
-        <v>37</v>
-      </c>
-      <c r="C12" s="16" t="s">
-        <v>129</v>
-      </c>
-      <c r="D12" s="16" t="s">
-        <v>130</v>
-      </c>
-      <c r="E12" s="16" t="s">
-        <v>131</v>
-      </c>
-      <c r="F12" s="16" t="s">
-        <v>132</v>
-      </c>
-      <c r="G12" s="16" t="s">
-        <v>8</v>
-      </c>
-      <c r="H12" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="I12" s="16">
-        <v>6</v>
-      </c>
-      <c r="J12" s="16" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="13" spans="2:10" ht="157.5" x14ac:dyDescent="0.25">
-      <c r="B13" s="16" t="s">
-        <v>38</v>
-      </c>
-      <c r="C13" s="16" t="s">
-        <v>133</v>
-      </c>
-      <c r="D13" s="16" t="s">
-        <v>134</v>
-      </c>
-      <c r="E13" s="16" t="s">
-        <v>135</v>
-      </c>
-      <c r="F13" s="16" t="s">
-        <v>86</v>
-      </c>
-      <c r="G13" s="16" t="s">
-        <v>8</v>
-      </c>
-      <c r="H13" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="I13" s="16">
-        <v>4</v>
-      </c>
-      <c r="J13" s="16" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="14" spans="2:10" ht="126" x14ac:dyDescent="0.25">
-      <c r="B14" s="16" t="s">
-        <v>136</v>
-      </c>
-      <c r="C14" s="16" t="s">
-        <v>137</v>
-      </c>
-      <c r="D14" s="16" t="s">
-        <v>138</v>
-      </c>
-      <c r="E14" s="16" t="s">
-        <v>139</v>
-      </c>
-      <c r="F14" s="16" t="s">
-        <v>91</v>
-      </c>
-      <c r="G14" s="16" t="s">
-        <v>8</v>
-      </c>
-      <c r="H14" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="I14" s="16">
-        <v>5</v>
-      </c>
-      <c r="J14" s="16" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="15" spans="2:10" ht="126" x14ac:dyDescent="0.25">
-      <c r="B15" s="16" t="s">
-        <v>140</v>
-      </c>
-      <c r="C15" s="16" t="s">
-        <v>141</v>
-      </c>
-      <c r="D15" s="16" t="s">
-        <v>142</v>
-      </c>
-      <c r="E15" s="16" t="s">
-        <v>143</v>
-      </c>
-      <c r="F15" s="16" t="s">
-        <v>100</v>
-      </c>
-      <c r="G15" s="16" t="s">
-        <v>20</v>
-      </c>
-      <c r="H15" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="I15" s="16">
-        <v>4</v>
-      </c>
-      <c r="J15" s="16" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="16" spans="2:10" ht="110.25" x14ac:dyDescent="0.25">
-      <c r="B16" s="16" t="s">
-        <v>144</v>
-      </c>
-      <c r="C16" s="16" t="s">
-        <v>145</v>
-      </c>
-      <c r="D16" s="16" t="s">
-        <v>146</v>
-      </c>
-      <c r="E16" s="16" t="s">
-        <v>147</v>
-      </c>
-      <c r="F16" s="16" t="s">
-        <v>98</v>
-      </c>
-      <c r="G16" s="16" t="s">
-        <v>20</v>
-      </c>
-      <c r="H16" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="I16" s="16">
-        <v>3</v>
-      </c>
-      <c r="J16" s="16" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="17" spans="2:10" ht="110.25" x14ac:dyDescent="0.25">
-      <c r="B17" s="16" t="s">
-        <v>148</v>
-      </c>
-      <c r="C17" s="16" t="s">
-        <v>149</v>
-      </c>
-      <c r="D17" s="16" t="s">
-        <v>150</v>
-      </c>
-      <c r="E17" s="16" t="s">
-        <v>151</v>
-      </c>
-      <c r="F17" s="16" t="s">
-        <v>106</v>
-      </c>
-      <c r="G17" s="16" t="s">
-        <v>8</v>
-      </c>
-      <c r="H17" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="I17" s="16">
-        <v>5</v>
-      </c>
-      <c r="J17" s="16" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="18" spans="2:10" ht="126" x14ac:dyDescent="0.25">
-      <c r="B18" s="16" t="s">
-        <v>152</v>
-      </c>
-      <c r="C18" s="16" t="s">
-        <v>153</v>
-      </c>
-      <c r="D18" s="16" t="s">
-        <v>154</v>
-      </c>
-      <c r="E18" s="16" t="s">
-        <v>155</v>
-      </c>
-      <c r="F18" s="16" t="s">
-        <v>106</v>
-      </c>
-      <c r="G18" s="16" t="s">
-        <v>8</v>
-      </c>
-      <c r="H18" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="I18" s="16">
-        <v>4</v>
-      </c>
-      <c r="J18" s="16" t="s">
+      <c r="J18" s="8" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="19" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B19" s="11" t="s">
+      <c r="B19" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="C19" s="12"/>
-      <c r="D19" s="12"/>
-      <c r="E19" s="12"/>
-      <c r="F19" s="12"/>
-      <c r="G19" s="12"/>
-      <c r="H19" s="13"/>
+      <c r="C19" s="13"/>
+      <c r="D19" s="13"/>
+      <c r="E19" s="13"/>
+      <c r="F19" s="13"/>
+      <c r="G19" s="13"/>
+      <c r="H19" s="14"/>
       <c r="I19" s="4">
         <f>SUM(I4:I18)</f>
         <v>61</v>
@@ -1884,548 +1890,548 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B2" s="10" t="s">
+      <c r="B2" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="10"/>
-      <c r="H2" s="10"/>
-      <c r="I2" s="10"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
+      <c r="H2" s="19"/>
+      <c r="I2" s="19"/>
     </row>
     <row r="3" spans="2:12" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="B3" s="15" t="s">
+      <c r="B3" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="15" t="s">
+      <c r="C3" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="D3" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="E3" s="15" t="s">
+      <c r="E3" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="F3" s="15" t="s">
+      <c r="F3" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="G3" s="15" t="s">
+      <c r="G3" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="H3" s="15" t="s">
+      <c r="H3" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="I3" s="15" t="s">
+      <c r="I3" s="7" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="4" spans="2:12" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="B4" s="16" t="s">
+      <c r="B4" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="C4" s="16" t="s">
+      <c r="C4" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="D4" s="16" t="s">
+      <c r="D4" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="E4" s="16" t="s">
+      <c r="E4" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="F4" s="16" t="s">
+      <c r="F4" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="G4" s="16" t="s">
-        <v>8</v>
-      </c>
-      <c r="H4" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="I4" s="16">
+      <c r="G4" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="I4" s="8">
         <v>3</v>
       </c>
     </row>
     <row r="5" spans="2:12" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="B5" s="16" t="s">
+      <c r="B5" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="16" t="s">
+      <c r="C5" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="D5" s="16" t="s">
+      <c r="D5" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="16" t="s">
+      <c r="E5" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="G5" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="H5" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="I5" s="8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="2:12" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="B6" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="G6" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="H6" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="I6" s="8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="2:12" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="B7" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="I7" s="8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="2:12" ht="63" x14ac:dyDescent="0.25">
+      <c r="B8" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="G8" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="H8" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="I8" s="8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="2:12" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="B9" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="G9" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="H9" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="I9" s="8">
+        <v>3</v>
+      </c>
+      <c r="L9" s="5"/>
+    </row>
+    <row r="10" spans="2:12" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B10" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="G10" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="H10" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="I10" s="8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="2:12" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B11" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="E11" s="8" t="s">
         <v>156</v>
       </c>
-      <c r="F5" s="16" t="s">
+      <c r="F11" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="G5" s="16" t="s">
-        <v>8</v>
-      </c>
-      <c r="H5" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="I5" s="16">
+      <c r="G11" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="H11" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="I11" s="8">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="2:12" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B12" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="G12" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="H12" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="I12" s="8">
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="2:12" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="B6" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="C6" s="16" t="s">
-        <v>54</v>
-      </c>
-      <c r="D6" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="E6" s="16" t="s">
+    <row r="13" spans="2:12" ht="78.75" x14ac:dyDescent="0.25">
+      <c r="B13" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="G13" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="H13" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="I13" s="8">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14" spans="2:12" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="B14" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="E14" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="G14" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="H14" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="I14" s="8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" spans="2:12" ht="94.5" x14ac:dyDescent="0.25">
+      <c r="B15" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E15" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="F6" s="16" t="s">
+      <c r="F15" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="G6" s="16" t="s">
-        <v>8</v>
-      </c>
-      <c r="H6" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="I6" s="16">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7" spans="2:12" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="B7" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="C7" s="16" t="s">
-        <v>54</v>
-      </c>
-      <c r="D7" s="16" t="s">
-        <v>30</v>
-      </c>
-      <c r="E7" s="16" t="s">
-        <v>107</v>
-      </c>
-      <c r="F7" s="16" t="s">
+      <c r="G15" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="H15" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="I15" s="8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="2:12" ht="63" x14ac:dyDescent="0.25">
+      <c r="B16" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="F16" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="G7" s="16" t="s">
-        <v>8</v>
-      </c>
-      <c r="H7" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="I7" s="16">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="8" spans="2:12" ht="63" x14ac:dyDescent="0.25">
-      <c r="B8" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="C8" s="16" t="s">
-        <v>54</v>
-      </c>
-      <c r="D8" s="16" t="s">
-        <v>31</v>
-      </c>
-      <c r="E8" s="16" t="s">
-        <v>110</v>
-      </c>
-      <c r="F8" s="16" t="s">
+      <c r="G16" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="H16" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="I16" s="8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="2:9" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="B17" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C17" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="D17" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="E17" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="F17" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="G8" s="16" t="s">
-        <v>8</v>
-      </c>
-      <c r="H8" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="I8" s="16">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="9" spans="2:12" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="B9" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="C9" s="16" t="s">
-        <v>54</v>
-      </c>
-      <c r="D9" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="E9" s="16" t="s">
-        <v>113</v>
-      </c>
-      <c r="F9" s="16" t="s">
+      <c r="G17" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="H17" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="I17" s="8">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18" spans="2:9" ht="63" x14ac:dyDescent="0.25">
+      <c r="B18" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="D18" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="F18" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="G9" s="16" t="s">
-        <v>8</v>
-      </c>
-      <c r="H9" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="I9" s="16">
-        <v>3</v>
-      </c>
-      <c r="L9" s="5"/>
-    </row>
-    <row r="10" spans="2:12" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="B10" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="C10" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="D10" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="E10" s="16" t="s">
-        <v>13</v>
-      </c>
-      <c r="F10" s="16" t="s">
+      <c r="G18" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="H18" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="I18" s="8">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="19" spans="2:9" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="B19" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C19" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D19" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="F19" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="G10" s="16" t="s">
-        <v>8</v>
-      </c>
-      <c r="H10" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="I10" s="16">
+      <c r="G19" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="H19" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="I19" s="8">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20" spans="2:9" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="B20" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D20" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="E20" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="F20" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="G20" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="H20" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="I20" s="8">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="21" spans="2:9" ht="63" x14ac:dyDescent="0.25">
+      <c r="B21" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C21" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D21" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="E21" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="F21" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="G21" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="H21" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="I21" s="8">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="22" spans="2:9" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="B22" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D22" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="E22" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="F22" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="G22" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="H22" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="I22" s="8">
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="2:12" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="B11" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="C11" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="D11" s="16" t="s">
-        <v>15</v>
-      </c>
-      <c r="E11" s="16" t="s">
-        <v>158</v>
-      </c>
-      <c r="F11" s="16" t="s">
-        <v>44</v>
-      </c>
-      <c r="G11" s="16" t="s">
-        <v>8</v>
-      </c>
-      <c r="H11" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="I11" s="16">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="12" spans="2:12" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="B12" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="C12" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="D12" s="16" t="s">
-        <v>17</v>
-      </c>
-      <c r="E12" s="16" t="s">
-        <v>16</v>
-      </c>
-      <c r="F12" s="16" t="s">
-        <v>44</v>
-      </c>
-      <c r="G12" s="16" t="s">
-        <v>8</v>
-      </c>
-      <c r="H12" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="I12" s="16">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="13" spans="2:12" ht="78.75" x14ac:dyDescent="0.25">
-      <c r="B13" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="C13" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="D13" s="16" t="s">
-        <v>33</v>
-      </c>
-      <c r="E13" s="16" t="s">
-        <v>116</v>
-      </c>
-      <c r="F13" s="16" t="s">
-        <v>43</v>
-      </c>
-      <c r="G13" s="16" t="s">
-        <v>8</v>
-      </c>
-      <c r="H13" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="I13" s="16">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="14" spans="2:12" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="B14" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="C14" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="D14" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="E14" s="16" t="s">
-        <v>120</v>
-      </c>
-      <c r="F14" s="16" t="s">
-        <v>43</v>
-      </c>
-      <c r="G14" s="16" t="s">
-        <v>8</v>
-      </c>
-      <c r="H14" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="I14" s="16">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="15" spans="2:12" ht="94.5" x14ac:dyDescent="0.25">
-      <c r="B15" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="C15" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="D15" s="16" t="s">
-        <v>19</v>
-      </c>
-      <c r="E15" s="16" t="s">
-        <v>159</v>
-      </c>
-      <c r="F15" s="16" t="s">
-        <v>44</v>
-      </c>
-      <c r="G15" s="16" t="s">
-        <v>8</v>
-      </c>
-      <c r="H15" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="I15" s="16">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="16" spans="2:12" ht="63" x14ac:dyDescent="0.25">
-      <c r="B16" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="C16" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="D16" s="16" t="s">
-        <v>35</v>
-      </c>
-      <c r="E16" s="16" t="s">
-        <v>160</v>
-      </c>
-      <c r="F16" s="16" t="s">
-        <v>43</v>
-      </c>
-      <c r="G16" s="16" t="s">
-        <v>8</v>
-      </c>
-      <c r="H16" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="I16" s="16">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="17" spans="2:9" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="B17" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="C17" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="D17" s="16" t="s">
-        <v>36</v>
-      </c>
-      <c r="E17" s="16" t="s">
-        <v>57</v>
-      </c>
-      <c r="F17" s="16" t="s">
-        <v>43</v>
-      </c>
-      <c r="G17" s="16" t="s">
-        <v>8</v>
-      </c>
-      <c r="H17" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="I17" s="16">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="18" spans="2:9" ht="63" x14ac:dyDescent="0.25">
-      <c r="B18" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="C18" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="D18" s="16" t="s">
-        <v>37</v>
-      </c>
-      <c r="E18" s="16" t="s">
-        <v>129</v>
-      </c>
-      <c r="F18" s="16" t="s">
-        <v>43</v>
-      </c>
-      <c r="G18" s="16" t="s">
-        <v>8</v>
-      </c>
-      <c r="H18" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="I18" s="16">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="19" spans="2:9" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="B19" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="C19" s="16" t="s">
-        <v>58</v>
-      </c>
-      <c r="D19" s="16" t="s">
-        <v>22</v>
-      </c>
-      <c r="E19" s="16" t="s">
-        <v>59</v>
-      </c>
-      <c r="F19" s="16" t="s">
-        <v>44</v>
-      </c>
-      <c r="G19" s="16" t="s">
-        <v>8</v>
-      </c>
-      <c r="H19" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="I19" s="16">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="20" spans="2:9" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="B20" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="C20" s="16" t="s">
-        <v>58</v>
-      </c>
-      <c r="D20" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="E20" s="16" t="s">
-        <v>23</v>
-      </c>
-      <c r="F20" s="16" t="s">
-        <v>44</v>
-      </c>
-      <c r="G20" s="16" t="s">
-        <v>8</v>
-      </c>
-      <c r="H20" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="I20" s="16">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="21" spans="2:9" ht="63" x14ac:dyDescent="0.25">
-      <c r="B21" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="C21" s="16" t="s">
-        <v>58</v>
-      </c>
-      <c r="D21" s="16" t="s">
-        <v>38</v>
-      </c>
-      <c r="E21" s="16" t="s">
-        <v>133</v>
-      </c>
-      <c r="F21" s="16" t="s">
-        <v>43</v>
-      </c>
-      <c r="G21" s="16" t="s">
-        <v>8</v>
-      </c>
-      <c r="H21" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="I21" s="16">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="22" spans="2:9" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="B22" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="C22" s="16" t="s">
-        <v>58</v>
-      </c>
-      <c r="D22" s="16" t="s">
-        <v>136</v>
-      </c>
-      <c r="E22" s="16" t="s">
-        <v>137</v>
-      </c>
-      <c r="F22" s="16" t="s">
-        <v>43</v>
-      </c>
-      <c r="G22" s="16" t="s">
-        <v>8</v>
-      </c>
-      <c r="H22" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="I22" s="16">
-        <v>5</v>
-      </c>
-    </row>
     <row r="23" spans="2:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B23" s="11" t="s">
+      <c r="B23" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="C23" s="12"/>
-      <c r="D23" s="12"/>
-      <c r="E23" s="12"/>
-      <c r="F23" s="12"/>
-      <c r="G23" s="12"/>
-      <c r="H23" s="13"/>
+      <c r="C23" s="13"/>
+      <c r="D23" s="13"/>
+      <c r="E23" s="13"/>
+      <c r="F23" s="13"/>
+      <c r="G23" s="13"/>
+      <c r="H23" s="14"/>
       <c r="I23" s="4">
         <f>SUM(I4:I22)</f>
         <v>82</v>

</xml_diff>